<commit_message>
Change cardinality of RetinaTiltaksstausForrigeUndersokelseExtension from 0..1 to 1..0 and update the examples Define and document optional observations for photo, OCT and  HbA1c in the diagnostic report profile Bump version to 0.1.3
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-no-kodeverk-8660.xlsx
+++ b/docs/CodeSystem-no-kodeverk-8660.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.2</t>
+    <t>0.1.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-19T20:08:40+02:00</t>
+    <t>2025-10-31T08:54:10+01:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>